<commit_message>
updates to work and test
</commit_message>
<xml_diff>
--- a/results_gen/outputs/Test_all.xlsx
+++ b/results_gen/outputs/Test_all.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reube\Parallel-Monte-Carlo-Tree-Search-For-The-Orienteering-Problem\results_gen\outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reubenkappely/Documents/Projects/Parallel-Monte-Carlo-Tree-Search-For-The-Orienteering-Problem/results_gen/outputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5351F0F-73B9-4227-89EA-B500E874AF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E99C3C2-967D-CD46-AE8E-616D3C4C354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-45" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{260B2045-1352-43BA-9B1E-29C2A8BE3BD5}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{260B2045-1352-43BA-9B1E-29C2A8BE3BD5}"/>
   </bookViews>
   <sheets>
     <sheet name="Test1" sheetId="1" r:id="rId1"/>
@@ -168,7 +168,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,6 +223,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -274,7 +281,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -334,11 +341,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -359,10 +397,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -371,16 +406,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -398,9 +433,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -736,50 +778,50 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2055FE3-E712-4367-9B42-B5E3B258A2F1}">
   <dimension ref="A1:V55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="41.5703125" customWidth="1"/>
+    <col min="1" max="1" width="41.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14" t="s">
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14" t="s">
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14" t="s">
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14" t="s">
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -842,7 +884,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -850,8 +892,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A6" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -867,8 +909,8 @@
         <v>376</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A7" s="20"/>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -885,8 +927,8 @@
         <v>390</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A8" s="20"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -903,8 +945,8 @@
         <v>388</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A9" s="20"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -921,8 +963,8 @@
         <v>358</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A10" s="20"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
@@ -939,8 +981,8 @@
         <v>395</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -956,8 +998,8 @@
         <v>558</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A12" s="15"/>
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
@@ -974,8 +1016,8 @@
         <v>526</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A13" s="15"/>
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
@@ -992,8 +1034,8 @@
         <v>509</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A14" s="15"/>
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
@@ -1010,8 +1052,8 @@
         <v>499</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A15" s="15"/>
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
@@ -1028,8 +1070,8 @@
         <v>501</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A16" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1045,8 +1087,8 @@
         <v>315</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="21"/>
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
@@ -1063,8 +1105,8 @@
         <v>350</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="22"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="21"/>
       <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1081,8 +1123,8 @@
         <v>332</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="21"/>
       <c r="B19" s="1" t="s">
         <v>11</v>
       </c>
@@ -1102,8 +1144,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="21"/>
       <c r="B20" s="1" t="s">
         <v>12</v>
       </c>
@@ -1120,8 +1162,8 @@
         <v>345</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
         <v>14</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1137,8 +1179,8 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="22"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="21"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -1155,8 +1197,8 @@
         <v>479</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="22"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="21"/>
       <c r="B23" s="1" t="s">
         <v>10</v>
       </c>
@@ -1173,8 +1215,8 @@
         <v>451</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="21"/>
       <c r="B24" s="1" t="s">
         <v>11</v>
       </c>
@@ -1191,8 +1233,8 @@
         <v>454</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="21"/>
       <c r="B25" s="1" t="s">
         <v>12</v>
       </c>
@@ -1209,14 +1251,14 @@
         <v>469</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C26" s="2">
         <v>453</v>
       </c>
       <c r="E26">
@@ -1226,8 +1268,8 @@
         <v>453</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="20"/>
       <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
@@ -1244,8 +1286,8 @@
         <v>486</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="20"/>
       <c r="B28" s="1" t="s">
         <v>10</v>
       </c>
@@ -1265,8 +1307,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="20"/>
       <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
@@ -1283,8 +1325,8 @@
         <v>465</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="20"/>
       <c r="B30" s="1" t="s">
         <v>12</v>
       </c>
@@ -1301,8 +1343,8 @@
         <v>480</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="15" t="s">
         <v>18</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -1318,8 +1360,8 @@
         <v>622</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="15"/>
       <c r="B32" s="1" t="s">
         <v>9</v>
       </c>
@@ -1336,8 +1378,8 @@
         <v>643</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A33" s="15"/>
       <c r="B33" s="1" t="s">
         <v>10</v>
       </c>
@@ -1354,8 +1396,8 @@
         <v>606</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A34" s="16"/>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A34" s="15"/>
       <c r="B34" s="1" t="s">
         <v>11</v>
       </c>
@@ -1372,8 +1414,8 @@
         <v>602</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A35" s="16"/>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A35" s="15"/>
       <c r="B35" s="1" t="s">
         <v>12</v>
       </c>
@@ -1390,8 +1432,8 @@
         <v>653</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A36" s="15" t="s">
         <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -1407,8 +1449,8 @@
         <v>414</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A37" s="16"/>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A37" s="15"/>
       <c r="B37" s="1" t="s">
         <v>9</v>
       </c>
@@ -1425,8 +1467,8 @@
         <v>380</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A38" s="16"/>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A38" s="15"/>
       <c r="B38" s="1" t="s">
         <v>10</v>
       </c>
@@ -1443,15 +1485,15 @@
         <v>390</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A39" s="15"/>
       <c r="B39" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C39">
         <v>321</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="29">
         <v>50.383529054642452</v>
       </c>
       <c r="E39">
@@ -1461,15 +1503,15 @@
         <v>390</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A40" s="15"/>
       <c r="B40" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C40">
         <v>308</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="29">
         <v>51.112620750652177</v>
       </c>
       <c r="E40">
@@ -1479,8 +1521,8 @@
         <v>392</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A41" s="15" t="s">
         <v>21</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -1496,8 +1538,8 @@
         <v>536</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A42" s="15"/>
       <c r="B42" s="1" t="s">
         <v>9</v>
       </c>
@@ -1514,8 +1556,8 @@
         <v>494</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A43" s="15"/>
       <c r="B43" s="1" t="s">
         <v>10</v>
       </c>
@@ -1532,8 +1574,8 @@
         <v>495</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A44" s="16"/>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A44" s="15"/>
       <c r="B44" s="1" t="s">
         <v>11</v>
       </c>
@@ -1550,8 +1592,8 @@
         <v>475</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A45" s="16"/>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A45" s="15"/>
       <c r="B45" s="1" t="s">
         <v>12</v>
       </c>
@@ -1568,14 +1610,14 @@
         <v>497</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A46" s="17" t="s">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A46" s="26" t="s">
         <v>23</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="5">
         <v>303</v>
       </c>
       <c r="E46">
@@ -1603,9 +1645,9 @@
         <v>99.621165057908925</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A47" s="18"/>
-      <c r="B47" s="27" t="s">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A47" s="27"/>
+      <c r="B47" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C47">
@@ -1669,8 +1711,8 @@
         <v>0.97419999999999995</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A48" s="18"/>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A48" s="27"/>
       <c r="B48" s="1" t="s">
         <v>10</v>
       </c>
@@ -1711,8 +1753,8 @@
         <v>99.329966244077795</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A49" s="19"/>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A49" s="27"/>
       <c r="B49" s="1" t="s">
         <v>11</v>
       </c>
@@ -1777,10 +1819,8 @@
         <v>0.54720000000000002</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A50" s="17" t="s">
-        <v>28</v>
-      </c>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A50" s="28"/>
       <c r="B50" s="1" t="s">
         <v>12</v>
       </c>
@@ -1821,12 +1861,14 @@
         <v>99.66498312203889</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A51" s="20"/>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A51" s="26" t="s">
+        <v>28</v>
+      </c>
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="5">
         <v>348</v>
       </c>
       <c r="E51">
@@ -1854,12 +1896,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A52" s="20"/>
-      <c r="B52" s="27" t="s">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A52" s="27"/>
+      <c r="B52" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="4">
         <v>443.6</v>
       </c>
       <c r="D52">
@@ -1920,8 +1962,8 @@
         <v>0.9829</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A53" s="21"/>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A53" s="27"/>
       <c r="B53" s="1" t="s">
         <v>10</v>
       </c>
@@ -1962,7 +2004,8 @@
         <v>99.497474683058343</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A54" s="27"/>
       <c r="B54" s="1" t="s">
         <v>11</v>
       </c>
@@ -2027,7 +2070,8 @@
         <v>0.69609999999999994</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A55" s="27"/>
       <c r="B55" s="1" t="s">
         <v>12</v>
       </c>
@@ -2070,11 +2114,7 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A31:A35"/>
-    <mergeCell ref="A36:A40"/>
-    <mergeCell ref="A41:A45"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="A51:A55"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="K3:N3"/>
     <mergeCell ref="O3:R3"/>
@@ -2085,6 +2125,10 @@
     <mergeCell ref="A11:A15"/>
     <mergeCell ref="A16:A20"/>
     <mergeCell ref="A21:A25"/>
+    <mergeCell ref="A31:A35"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="A41:A45"/>
+    <mergeCell ref="A46:A50"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2093,51 +2137,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B9F7C1-6CD3-4B61-9368-31485E040906}">
   <dimension ref="A1:V55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14" t="s">
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14" t="s">
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14" t="s">
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14" t="s">
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -2200,7 +2244,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -2208,8 +2252,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A6" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -2225,8 +2269,8 @@
         <v>376</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A7" s="20"/>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -2243,8 +2287,8 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A8" s="20"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -2261,8 +2305,8 @@
         <v>379</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A9" s="20"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -2279,8 +2323,8 @@
         <v>417</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A10" s="20"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
@@ -2297,8 +2341,8 @@
         <v>404</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -2314,8 +2358,8 @@
         <v>558</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A12" s="15"/>
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
@@ -2335,8 +2379,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A13" s="15"/>
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
@@ -2353,8 +2397,8 @@
         <v>503</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A14" s="15"/>
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
@@ -2371,12 +2415,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A15" s="15"/>
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="3">
         <v>498.4</v>
       </c>
       <c r="D15">
@@ -2389,8 +2433,8 @@
         <v>518</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A16" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -2406,8 +2450,8 @@
         <v>315</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="21"/>
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
@@ -2424,8 +2468,8 @@
         <v>352</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="22"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="21"/>
       <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
@@ -2442,8 +2486,8 @@
         <v>345</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="21"/>
       <c r="B19" s="1" t="s">
         <v>11</v>
       </c>
@@ -2460,8 +2504,8 @@
         <v>339</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="26"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="25"/>
       <c r="B20" s="8" t="s">
         <v>12</v>
       </c>
@@ -2478,8 +2522,8 @@
         <v>345</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="17" t="s">
         <v>14</v>
       </c>
       <c r="B21" s="9" t="s">
@@ -2495,8 +2539,8 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="20"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="17"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -2513,8 +2557,8 @@
         <v>434</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="20"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="17"/>
       <c r="B23" s="1" t="s">
         <v>10</v>
       </c>
@@ -2531,8 +2575,8 @@
         <v>453</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="20"/>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="17"/>
       <c r="B24" s="1" t="s">
         <v>11</v>
       </c>
@@ -2549,8 +2593,8 @@
         <v>416</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="21"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="18"/>
       <c r="B25" s="1" t="s">
         <v>12</v>
       </c>
@@ -2567,8 +2611,8 @@
         <v>481</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="17" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="16" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -2584,8 +2628,8 @@
         <v>453</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="20"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="17"/>
       <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
@@ -2605,8 +2649,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="20"/>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="17"/>
       <c r="B28" s="1" t="s">
         <v>10</v>
       </c>
@@ -2623,8 +2667,8 @@
         <v>481</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="20"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="17"/>
       <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
@@ -2641,8 +2685,8 @@
         <v>495</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="21"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="18"/>
       <c r="B30" s="1" t="s">
         <v>12</v>
       </c>
@@ -2659,8 +2703,8 @@
         <v>510</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="23" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="22" t="s">
         <v>18</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -2676,8 +2720,8 @@
         <v>622</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="24"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="23"/>
       <c r="B32" s="1" t="s">
         <v>9</v>
       </c>
@@ -2694,8 +2738,8 @@
         <v>608</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A33" s="24"/>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A33" s="23"/>
       <c r="B33" s="1" t="s">
         <v>10</v>
       </c>
@@ -2712,8 +2756,8 @@
         <v>610</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A34" s="24"/>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A34" s="23"/>
       <c r="B34" s="1" t="s">
         <v>11</v>
       </c>
@@ -2730,12 +2774,12 @@
         <v>625</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A35" s="25"/>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A35" s="24"/>
       <c r="B35" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="3">
         <v>592</v>
       </c>
       <c r="D35">
@@ -2748,8 +2792,8 @@
         <v>643</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A36" s="23" t="s">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A36" s="22" t="s">
         <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -2765,8 +2809,8 @@
         <v>414</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A37" s="24"/>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A37" s="23"/>
       <c r="B37" s="1" t="s">
         <v>9</v>
       </c>
@@ -2786,8 +2830,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A38" s="24"/>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A38" s="23"/>
       <c r="B38" s="1" t="s">
         <v>10</v>
       </c>
@@ -2804,8 +2848,8 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A39" s="24"/>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A39" s="23"/>
       <c r="B39" s="1" t="s">
         <v>11</v>
       </c>
@@ -2822,8 +2866,8 @@
         <v>378</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A40" s="25"/>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A40" s="24"/>
       <c r="B40" s="1" t="s">
         <v>12</v>
       </c>
@@ -2840,8 +2884,8 @@
         <v>309</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A41" s="23" t="s">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A41" s="22" t="s">
         <v>21</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -2857,8 +2901,8 @@
         <v>536</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A42" s="24"/>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A42" s="23"/>
       <c r="B42" s="1" t="s">
         <v>9</v>
       </c>
@@ -2875,8 +2919,8 @@
         <v>497</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A43" s="24"/>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A43" s="23"/>
       <c r="B43" s="1" t="s">
         <v>10</v>
       </c>
@@ -2896,8 +2940,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A44" s="24"/>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A44" s="23"/>
       <c r="B44" s="1" t="s">
         <v>11</v>
       </c>
@@ -2914,8 +2958,8 @@
         <v>432</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A45" s="25"/>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A45" s="24"/>
       <c r="B45" s="1" t="s">
         <v>12</v>
       </c>
@@ -2932,8 +2976,8 @@
         <v>454</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A46" s="17" t="s">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A46" s="16" t="s">
         <v>23</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -2967,8 +3011,8 @@
         <v>99.621165057908925</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A47" s="20"/>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A47" s="17"/>
       <c r="B47" s="1" t="s">
         <v>9</v>
       </c>
@@ -3033,8 +3077,8 @@
         <v>0.98160000000000003</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A48" s="20"/>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A48" s="17"/>
       <c r="B48" s="1" t="s">
         <v>10</v>
       </c>
@@ -3075,8 +3119,8 @@
         <v>99.329966244077795</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A49" s="20"/>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A49" s="17"/>
       <c r="B49" s="1" t="s">
         <v>11</v>
       </c>
@@ -3141,8 +3185,8 @@
         <v>0.89880000000000004</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A50" s="21"/>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A50" s="18"/>
       <c r="B50" s="1" t="s">
         <v>12</v>
       </c>
@@ -3183,8 +3227,8 @@
         <v>99.66498312203889</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A51" s="17" t="s">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A51" s="16" t="s">
         <v>28</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -3218,8 +3262,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A52" s="20"/>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A52" s="17"/>
       <c r="B52" s="1" t="s">
         <v>9</v>
       </c>
@@ -3284,8 +3328,8 @@
         <v>0.88500000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A53" s="20"/>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A53" s="17"/>
       <c r="B53" s="1" t="s">
         <v>10</v>
       </c>
@@ -3326,8 +3370,8 @@
         <v>99.497474683058343</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A54" s="20"/>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A54" s="17"/>
       <c r="B54" s="1" t="s">
         <v>11</v>
       </c>
@@ -3392,8 +3436,8 @@
         <v>0.89949999999999997</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A55" s="21"/>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A55" s="18"/>
       <c r="B55" s="1" t="s">
         <v>12</v>
       </c>
@@ -3459,51 +3503,51 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58126609-257A-4A45-B385-DFB3BFE448A7}">
   <dimension ref="A1:V55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14" t="s">
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14" t="s">
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14" t="s">
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14" t="s">
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -3566,7 +3610,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -3574,8 +3618,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A6" s="21" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -3591,8 +3635,8 @@
         <v>376</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" s="22"/>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A7" s="21"/>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -3609,8 +3653,8 @@
         <v>398</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A8" s="22"/>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A8" s="21"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -3627,8 +3671,8 @@
         <v>393</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A9" s="21"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -3645,8 +3689,8 @@
         <v>392</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A10" s="21"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
@@ -3663,8 +3707,8 @@
         <v>401</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A11" s="15" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -3680,8 +3724,8 @@
         <v>558</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A12" s="15"/>
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
@@ -3698,8 +3742,8 @@
         <v>534</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A13" s="15"/>
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
@@ -3716,8 +3760,8 @@
         <v>496</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A14" s="15"/>
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
@@ -3734,8 +3778,8 @@
         <v>508</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A15" s="15"/>
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
@@ -3752,8 +3796,8 @@
         <v>518</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A16" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -3769,8 +3813,8 @@
         <v>315</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="21"/>
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
@@ -3787,8 +3831,8 @@
         <v>350</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="22"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="21"/>
       <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
@@ -3808,8 +3852,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="21"/>
       <c r="B19" s="1" t="s">
         <v>11</v>
       </c>
@@ -3826,8 +3870,8 @@
         <v>354</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="21"/>
       <c r="B20" s="1" t="s">
         <v>12</v>
       </c>
@@ -3844,8 +3888,8 @@
         <v>353</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
         <v>14</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -3861,8 +3905,8 @@
         <v>444</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="22"/>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="21"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -3879,8 +3923,8 @@
         <v>463</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="22"/>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="21"/>
       <c r="B23" s="1" t="s">
         <v>10</v>
       </c>
@@ -3897,8 +3941,8 @@
         <v>451</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="21"/>
       <c r="B24" s="1" t="s">
         <v>11</v>
       </c>
@@ -3915,8 +3959,8 @@
         <v>401</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="21"/>
       <c r="B25" s="1" t="s">
         <v>12</v>
       </c>
@@ -3933,8 +3977,8 @@
         <v>434</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -3950,8 +3994,8 @@
         <v>453</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="20"/>
       <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
@@ -3968,8 +4012,8 @@
         <v>515</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="20"/>
       <c r="B28" s="1" t="s">
         <v>10</v>
       </c>
@@ -3986,8 +4030,8 @@
         <v>477</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="20"/>
       <c r="B29" s="1" t="s">
         <v>11</v>
       </c>
@@ -4004,8 +4048,8 @@
         <v>475</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="20"/>
       <c r="B30" s="1" t="s">
         <v>12</v>
       </c>
@@ -4022,8 +4066,8 @@
         <v>535</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="15" t="s">
         <v>18</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -4039,8 +4083,8 @@
         <v>622</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="15"/>
       <c r="B32" s="1" t="s">
         <v>9</v>
       </c>
@@ -4057,8 +4101,8 @@
         <v>615</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A33" s="15"/>
       <c r="B33" s="1" t="s">
         <v>10</v>
       </c>
@@ -4075,8 +4119,8 @@
         <v>598</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A34" s="16"/>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A34" s="15"/>
       <c r="B34" s="1" t="s">
         <v>11</v>
       </c>
@@ -4093,8 +4137,8 @@
         <v>584</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A35" s="16"/>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A35" s="15"/>
       <c r="B35" s="1" t="s">
         <v>12</v>
       </c>
@@ -4111,8 +4155,8 @@
         <v>620</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A36" s="15" t="s">
         <v>20</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -4128,8 +4172,8 @@
         <v>414</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A37" s="16"/>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A37" s="15"/>
       <c r="B37" s="1" t="s">
         <v>9</v>
       </c>
@@ -4146,8 +4190,8 @@
         <v>397</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A38" s="16"/>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A38" s="15"/>
       <c r="B38" s="1" t="s">
         <v>10</v>
       </c>
@@ -4164,8 +4208,8 @@
         <v>383</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A39" s="16"/>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A39" s="15"/>
       <c r="B39" s="1" t="s">
         <v>11</v>
       </c>
@@ -4182,8 +4226,8 @@
         <v>362</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A40" s="16"/>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A40" s="15"/>
       <c r="B40" s="1" t="s">
         <v>12</v>
       </c>
@@ -4200,8 +4244,8 @@
         <v>379</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A41" s="15" t="s">
         <v>21</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -4217,8 +4261,8 @@
         <v>536</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A42" s="16"/>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A42" s="15"/>
       <c r="B42" s="1" t="s">
         <v>9</v>
       </c>
@@ -4235,8 +4279,8 @@
         <v>483</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A43" s="15"/>
       <c r="B43" s="1" t="s">
         <v>10</v>
       </c>
@@ -4253,8 +4297,8 @@
         <v>476</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A44" s="16"/>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A44" s="15"/>
       <c r="B44" s="1" t="s">
         <v>11</v>
       </c>
@@ -4271,8 +4315,8 @@
         <v>479</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A45" s="16"/>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A45" s="15"/>
       <c r="B45" s="1" t="s">
         <v>12</v>
       </c>
@@ -4289,8 +4333,8 @@
         <v>463</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A46" s="15" t="s">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A46" s="20" t="s">
         <v>23</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -4324,9 +4368,9 @@
         <v>99.621165057908925</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
-      <c r="B47" s="27" t="s">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A47" s="20"/>
+      <c r="B47" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C47">
@@ -4390,8 +4434,8 @@
         <v>0.99695999999999996</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A48" s="20"/>
       <c r="B48" s="1" t="s">
         <v>10</v>
       </c>
@@ -4432,8 +4476,8 @@
         <v>99.66498312203889</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A49" s="20"/>
       <c r="B49" s="1" t="s">
         <v>11</v>
       </c>
@@ -4498,8 +4542,8 @@
         <v>0.89973999999999998</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A50" s="15" t="s">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A50" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -4542,8 +4586,8 @@
         <v>99.66498312203889</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A51" s="15"/>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A51" s="20"/>
       <c r="B51" s="1" t="s">
         <v>8</v>
       </c>
@@ -4575,9 +4619,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A52" s="15"/>
-      <c r="B52" s="27" t="s">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A52" s="20"/>
+      <c r="B52" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C52">
@@ -4641,8 +4685,8 @@
         <v>0.98977999999999999</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A53" s="15"/>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A53" s="20"/>
       <c r="B53" s="1" t="s">
         <v>10</v>
       </c>
@@ -4683,7 +4727,7 @@
         <v>99.497474683058343</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B54" s="1" t="s">
         <v>11</v>
       </c>
@@ -4748,7 +4792,7 @@
         <v>0.87141999999999997</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B55" s="1" t="s">
         <v>12</v>
       </c>
@@ -4791,6 +4835,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="O3:R3"/>
+    <mergeCell ref="S3:V3"/>
+    <mergeCell ref="A31:A35"/>
+    <mergeCell ref="A36:A40"/>
     <mergeCell ref="A41:A45"/>
     <mergeCell ref="A46:A49"/>
     <mergeCell ref="A50:A53"/>
@@ -4801,11 +4850,6 @@
     <mergeCell ref="A16:A20"/>
     <mergeCell ref="A21:A25"/>
     <mergeCell ref="A26:A30"/>
-    <mergeCell ref="K3:N3"/>
-    <mergeCell ref="O3:R3"/>
-    <mergeCell ref="S3:V3"/>
-    <mergeCell ref="A31:A35"/>
-    <mergeCell ref="A36:A40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4814,51 +4858,51 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986CE34A-0472-4CC3-8683-488EBE5AEA7F}">
   <dimension ref="A1:V25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14" t="s">
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14" t="s">
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14" t="s">
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14" t="s">
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -4921,7 +4965,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -4929,8 +4973,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A6" s="15" t="s">
         <v>33</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -4964,8 +5008,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A7" s="15"/>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -5030,8 +5074,8 @@
         <v>0.99913006959443251</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A8" s="15"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -5072,8 +5116,8 @@
         <v>99.859822611795806</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A9" s="15"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -5138,8 +5182,8 @@
         <v>0.98155994514318612</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A10" s="15"/>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
@@ -5180,8 +5224,8 @@
         <v>99.97947149678194</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A11" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -5215,8 +5259,8 @@
         <v>99.815513037361498</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A12" s="20"/>
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
@@ -5281,8 +5325,8 @@
         <v>0.9956803455723543</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A13" s="15"/>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A13" s="20"/>
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
@@ -5323,8 +5367,8 @@
         <v>99.949805167498852</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A14" s="15"/>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A14" s="20"/>
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
@@ -5389,8 +5433,8 @@
         <v>0.9741402003092362</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A15" s="20"/>
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
@@ -5431,8 +5475,8 @@
         <v>99.905041124119734</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A16" s="15" t="s">
         <v>35</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -5466,8 +5510,8 @@
         <v>99.402258737115403</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A17" s="15"/>
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
@@ -5532,8 +5576,8 @@
         <v>0.9962702983761299</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A18" s="15"/>
       <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
@@ -5574,8 +5618,8 @@
         <v>99.77729176583685</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A19" s="15"/>
       <c r="B19" s="1" t="s">
         <v>11</v>
       </c>
@@ -5640,12 +5684,12 @@
         <v>0.9773601083232194</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A20" s="15"/>
       <c r="B20" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="4">
         <v>1273.4000000000001</v>
       </c>
       <c r="D20" s="10">
@@ -5682,8 +5726,8 @@
         <v>99.879847952967822</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A21" s="15" t="s">
         <v>36</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -5717,8 +5761,8 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A22" s="15"/>
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
@@ -5783,8 +5827,8 @@
         <v>0.993960483161347</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A23" s="15"/>
       <c r="B23" s="1" t="s">
         <v>10</v>
       </c>
@@ -5816,8 +5860,8 @@
         <v>99.790140317807797</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A24" s="15"/>
       <c r="B24" s="1" t="s">
         <v>11</v>
       </c>
@@ -5882,8 +5926,8 @@
         <v>0.96782992270014778</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A25" s="15"/>
       <c r="B25" s="1" t="s">
         <v>12</v>
       </c>
@@ -5926,15 +5970,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="O3:R3"/>
+    <mergeCell ref="S3:V3"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="A6:A10"/>
     <mergeCell ref="A11:A15"/>
     <mergeCell ref="A16:A20"/>
     <mergeCell ref="A21:A25"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="K3:N3"/>
-    <mergeCell ref="O3:R3"/>
-    <mergeCell ref="S3:V3"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="A6:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>